<commit_message>
Add cartridge/sensor builder to Concept B configurator
Adopt the sensor-selection concept from the USD Purchase/Lease price list:
build a multi-gas cartridge by picking individual sensors, priced on the
rental sensor tiers.

- New 'Cartridge & sensors' section on Build a Kit: cartridge type
  (diffusion/pumped), combustible LEL (LEL-IR/LEL-MPS), oxygen (O2), and two
  toxic sensor slots the user picks from the full gas list.
- Sensor pricing by rental tier: standard sensors (LEL/O2/H2S/CO/SO2) included
  in the cartridge; Premium +/day, CO2 +0/day, PID/HF +5/day (pre-discount).
- Menu tab gains a SensorMap (sensor -> tier SKU) so each pick resolves to a
  Price List rate; prices stay single-sourced.
- README documents the sensor builder and tier table.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VPwdzhCqdwUCiCMnXPwJ7W
</commit_message>
<xml_diff>
--- a/Rental_Kit_Configurator.xlsx
+++ b/Rental_Kit_Configurator.xlsx
@@ -128,11 +128,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30"/>
-    <col min="2" max="2" width="52"/>
+    <col min="2" max="2" width="46"/>
     <col min="3" max="3" width="26"/>
     <col min="4" max="4" width="11"/>
     <col min="5" max="5" width="8"/>
@@ -150,7 +150,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Configure one kit below, set how many kits and how many days — the bundle prices itself.</t>
+          <t xml:space="preserve">Configure one kit (device + cartridge + sensors + add-ons), then set how many kits and days.</t>
         </is>
       </c>
     </row>
@@ -165,7 +165,7 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">(0 / 0.10 / 0.15 / 0.20 / 0.25 — applies to discountable items)</t>
+          <t xml:space="preserve">(0 / 0.10 / 0.15 / 0.20 / 0.25 - applies to discountable items)</t>
         </is>
       </c>
     </row>
@@ -204,12 +204,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Item  (pick from menu)</t>
+          <t xml:space="preserve">Item / sensor  (pick from menu)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SKU</t>
+          <t xml:space="preserve">SKU / tier</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -259,12 +259,12 @@
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 - Sensors &amp; cartridges</t>
+          <t xml:space="preserve">2 - Cartridge &amp; sensors</t>
         </is>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="8">
-        <f>IFERROR(VLOOKUP($B10,Menu!$A:$B,2,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP($B10,Menu!$Q:$R,2,FALSE),"")</f>
       </c>
       <c r="D10" s="3">
         <f>IF($C10="","",IFERROR(VLOOKUP($C10,'Price List'!$A:$E,4,FALSE),""))</f>
@@ -282,12 +282,12 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">  - Combustible (LEL)</t>
         </is>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="8">
-        <f>IFERROR(VLOOKUP($B11,Menu!$A:$B,2,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP($B11,Menu!$Q:$R,2,FALSE),"")</f>
       </c>
       <c r="D11" s="3">
         <f>IF($C11="","",IFERROR(VLOOKUP($C11,'Price List'!$A:$E,4,FALSE),""))</f>
@@ -305,12 +305,12 @@
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 - EXO modules &amp; accessories</t>
+          <t xml:space="preserve">  - Oxygen</t>
         </is>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="8">
-        <f>IFERROR(VLOOKUP($B12,Menu!$A:$B,2,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP($B12,Menu!$Q:$R,2,FALSE),"")</f>
       </c>
       <c r="D12" s="3">
         <f>IF($C12="","",IFERROR(VLOOKUP($C12,'Price List'!$A:$E,4,FALSE),""))</f>
@@ -328,12 +328,12 @@
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">  - Toxic sensor #1</t>
         </is>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="8">
-        <f>IFERROR(VLOOKUP($B13,Menu!$A:$B,2,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP($B13,Menu!$Q:$R,2,FALSE),"")</f>
       </c>
       <c r="D13" s="3">
         <f>IF($C13="","",IFERROR(VLOOKUP($C13,'Price List'!$A:$E,4,FALSE),""))</f>
@@ -351,12 +351,12 @@
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 - Docking, charging &amp; G7 accessories</t>
+          <t xml:space="preserve">  - Toxic sensor #2</t>
         </is>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="8">
-        <f>IFERROR(VLOOKUP($B14,Menu!$A:$B,2,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP($B14,Menu!$Q:$R,2,FALSE),"")</f>
       </c>
       <c r="D14" s="3">
         <f>IF($C14="","",IFERROR(VLOOKUP($C14,'Price List'!$A:$E,4,FALSE),""))</f>
@@ -374,7 +374,7 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">3 - EXO modules &amp; accessories</t>
         </is>
       </c>
       <c r="B15" s="4"/>
@@ -420,7 +420,7 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 - G6 accessories &amp; docks</t>
+          <t xml:space="preserve">4 - Docking, charging &amp; G7 accessories</t>
         </is>
       </c>
       <c r="B17" s="4"/>
@@ -466,7 +466,7 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 - Monitoring &amp; data plans</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="B19" s="4"/>
@@ -489,7 +489,7 @@
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">5 - G6 accessories &amp; docks</t>
         </is>
       </c>
       <c r="B20" s="4"/>
@@ -535,7 +535,7 @@
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">7 - Gas cylinders &amp; consumables</t>
+          <t xml:space="preserve">6 - Monitoring &amp; data plans</t>
         </is>
       </c>
       <c r="B22" s="4"/>
@@ -602,167 +602,236 @@
       </c>
     </row>
     <row r="25">
-      <c r="E25" s="0" t="inlineStr">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7 - Gas cylinders &amp; consumables</t>
+        </is>
+      </c>
+      <c r="B25" s="4"/>
+      <c r="C25" s="8">
+        <f>IFERROR(VLOOKUP($B25,Menu!$A:$B,2,FALSE),"")</f>
+      </c>
+      <c r="D25" s="3">
+        <f>IF($C25="","",IFERROR(VLOOKUP($C25,'Price List'!$A:$E,4,FALSE),""))</f>
+      </c>
+      <c r="E25" s="13">
+        <v>1</v>
+      </c>
+      <c r="F25" s="3">
+        <f>IF($C25="","",$D25*(1-IF(IFERROR(VLOOKUP($C25,'Price List'!$A:$E,5,FALSE),0)=1,$C$3,0)))</f>
+      </c>
+      <c r="G25" s="3">
+        <f>IF(OR($C25="",$E25=""),0,$F25*$E25)</f>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="F25" s="11" t="inlineStr">
+      <c r="B26" s="4"/>
+      <c r="C26" s="8">
+        <f>IFERROR(VLOOKUP($B26,Menu!$A:$B,2,FALSE),"")</f>
+      </c>
+      <c r="D26" s="3">
+        <f>IF($C26="","",IFERROR(VLOOKUP($C26,'Price List'!$A:$E,4,FALSE),""))</f>
+      </c>
+      <c r="E26" s="13">
+        <v>1</v>
+      </c>
+      <c r="F26" s="3">
+        <f>IF($C26="","",$D26*(1-IF(IFERROR(VLOOKUP($C26,'Price List'!$A:$E,5,FALSE),0)=1,$C$3,0)))</f>
+      </c>
+      <c r="G26" s="3">
+        <f>IF(OR($C26="",$E26=""),0,$F26*$E26)</f>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B27" s="4"/>
+      <c r="C27" s="8">
+        <f>IFERROR(VLOOKUP($B27,Menu!$A:$B,2,FALSE),"")</f>
+      </c>
+      <c r="D27" s="3">
+        <f>IF($C27="","",IFERROR(VLOOKUP($C27,'Price List'!$A:$E,4,FALSE),""))</f>
+      </c>
+      <c r="E27" s="13">
+        <v>1</v>
+      </c>
+      <c r="F27" s="3">
+        <f>IF($C27="","",$D27*(1-IF(IFERROR(VLOOKUP($C27,'Price List'!$A:$E,5,FALSE),0)=1,$C$3,0)))</f>
+      </c>
+      <c r="G27" s="3">
+        <f>IF(OR($C27="",$E27=""),0,$F27*$E27)</f>
+      </c>
+    </row>
+    <row r="28">
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">Kit subtotal / day</t>
         </is>
       </c>
-      <c r="G25" s="7">
-        <f>SUM(G9:G24)</f>
-      </c>
-    </row>
-    <row r="26">
-      <c r="F26" s="11" t="inlineStr">
+      <c r="G28" s="7">
+        <f>SUM(G9:G27)</f>
+      </c>
+    </row>
+    <row r="29">
+      <c r="F29" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">KIT TOTAL  (x kits x days)</t>
         </is>
       </c>
-      <c r="G26" s="7">
-        <f>G25*$C$4*$C$5</f>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="1" t="inlineStr">
+      <c r="G29" s="7">
+        <f>G28*$C$4*$C$5</f>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">One-time services  (charged once, not per day)</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Section</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Item  (pick from menu)</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">SKU</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Each</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Qty</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Your price</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Total</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">One-time</t>
         </is>
       </c>
-      <c r="B30" s="4"/>
-      <c r="C30" s="8">
-        <f>IFERROR(VLOOKUP($B30,Menu!$A:$B,2,FALSE),"")</f>
-      </c>
-      <c r="D30" s="3">
-        <f>IF($C30="","",IFERROR(VLOOKUP($C30,'Price List'!$A:$E,4,FALSE),""))</f>
-      </c>
-      <c r="E30" s="13">
-        <v>1</v>
-      </c>
-      <c r="F30" s="3">
-        <f>IF($C30="","",$D30*(1-IF(IFERROR(VLOOKUP($C30,'Price List'!$A:$E,5,FALSE),0)=1,$C$3,0)))</f>
-      </c>
-      <c r="G30" s="3">
-        <f>IF(OR($C30="",$E30=""),0,$F30*$E30)</f>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="12" t="inlineStr">
+      <c r="B33" s="4"/>
+      <c r="C33" s="8">
+        <f>IFERROR(VLOOKUP($B33,Menu!$A:$B,2,FALSE),"")</f>
+      </c>
+      <c r="D33" s="3">
+        <f>IF($C33="","",IFERROR(VLOOKUP($C33,'Price List'!$A:$E,4,FALSE),""))</f>
+      </c>
+      <c r="E33" s="13">
+        <v>1</v>
+      </c>
+      <c r="F33" s="3">
+        <f>IF($C33="","",$D33*(1-IF(IFERROR(VLOOKUP($C33,'Price List'!$A:$E,5,FALSE),0)=1,$C$3,0)))</f>
+      </c>
+      <c r="G33" s="3">
+        <f>IF(OR($C33="",$E33=""),0,$F33*$E33)</f>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="B31" s="4"/>
-      <c r="C31" s="8">
-        <f>IFERROR(VLOOKUP($B31,Menu!$A:$B,2,FALSE),"")</f>
-      </c>
-      <c r="D31" s="3">
-        <f>IF($C31="","",IFERROR(VLOOKUP($C31,'Price List'!$A:$E,4,FALSE),""))</f>
-      </c>
-      <c r="E31" s="13">
-        <v>1</v>
-      </c>
-      <c r="F31" s="3">
-        <f>IF($C31="","",$D31*(1-IF(IFERROR(VLOOKUP($C31,'Price List'!$A:$E,5,FALSE),0)=1,$C$3,0)))</f>
-      </c>
-      <c r="G31" s="3">
-        <f>IF(OR($C31="",$E31=""),0,$F31*$E31)</f>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="12" t="inlineStr">
+      <c r="B34" s="4"/>
+      <c r="C34" s="8">
+        <f>IFERROR(VLOOKUP($B34,Menu!$A:$B,2,FALSE),"")</f>
+      </c>
+      <c r="D34" s="3">
+        <f>IF($C34="","",IFERROR(VLOOKUP($C34,'Price List'!$A:$E,4,FALSE),""))</f>
+      </c>
+      <c r="E34" s="13">
+        <v>1</v>
+      </c>
+      <c r="F34" s="3">
+        <f>IF($C34="","",$D34*(1-IF(IFERROR(VLOOKUP($C34,'Price List'!$A:$E,5,FALSE),0)=1,$C$3,0)))</f>
+      </c>
+      <c r="G34" s="3">
+        <f>IF(OR($C34="",$E34=""),0,$F34*$E34)</f>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="B32" s="4"/>
-      <c r="C32" s="8">
-        <f>IFERROR(VLOOKUP($B32,Menu!$A:$B,2,FALSE),"")</f>
-      </c>
-      <c r="D32" s="3">
-        <f>IF($C32="","",IFERROR(VLOOKUP($C32,'Price List'!$A:$E,4,FALSE),""))</f>
-      </c>
-      <c r="E32" s="13">
-        <v>1</v>
-      </c>
-      <c r="F32" s="3">
-        <f>IF($C32="","",$D32*(1-IF(IFERROR(VLOOKUP($C32,'Price List'!$A:$E,5,FALSE),0)=1,$C$3,0)))</f>
-      </c>
-      <c r="G32" s="3">
-        <f>IF(OR($C32="",$E32=""),0,$F32*$E32)</f>
-      </c>
-    </row>
-    <row r="33">
-      <c r="F33" s="11" t="inlineStr">
+      <c r="B35" s="4"/>
+      <c r="C35" s="8">
+        <f>IFERROR(VLOOKUP($B35,Menu!$A:$B,2,FALSE),"")</f>
+      </c>
+      <c r="D35" s="3">
+        <f>IF($C35="","",IFERROR(VLOOKUP($C35,'Price List'!$A:$E,4,FALSE),""))</f>
+      </c>
+      <c r="E35" s="13">
+        <v>1</v>
+      </c>
+      <c r="F35" s="3">
+        <f>IF($C35="","",$D35*(1-IF(IFERROR(VLOOKUP($C35,'Price List'!$A:$E,5,FALSE),0)=1,$C$3,0)))</f>
+      </c>
+      <c r="G35" s="3">
+        <f>IF(OR($C35="",$E35=""),0,$F35*$E35)</f>
+      </c>
+    </row>
+    <row r="36">
+      <c r="F36" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">One-time subtotal</t>
         </is>
       </c>
-      <c r="G33" s="7">
-        <f>SUM(G30:G32)</f>
-      </c>
-    </row>
-    <row r="35">
-      <c r="F35" s="11" t="inlineStr">
+      <c r="G36" s="7">
+        <f>SUM(G33:G35)</f>
+      </c>
+    </row>
+    <row r="38">
+      <c r="F38" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">GRAND TOTAL</t>
         </is>
       </c>
-      <c r="G35" s="7">
-        <f>G26+G33</f>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tip: use the Quote tool (Concept A) for free-form line items; this tab is for standardized kits. Edit prices on the Price List tab.</t>
+      <c r="G38" s="7">
+        <f>G29+G36</f>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sensors: standard sensors (LEL, O2, H2S, CO, SO2) are included in the cartridge. Premium = +$4/day list, CO2 = +$10/day, PID/HF = +$15/day (before discount).</t>
         </is>
       </c>
     </row>
@@ -771,33 +840,45 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
   </mergeCells>
-  <dataValidations count="9">
+  <dataValidations count="13">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C3">
       <formula1>"0,0.1,0.15,0.2,0.25"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B9:B9">
       <formula1>Menu!$D$2:$D$15</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10:B11">
-      <formula1>Menu!$E$2:$E$7</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10:B10">
+      <formula1>Menu!$L$2:$L$4</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B12:B13">
-      <formula1>Menu!$F$2:$F$25</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B11:B11">
+      <formula1>Menu!$M$2:$M$4</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B14:B16">
-      <formula1>Menu!$G$2:$G$13</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B12:B12">
+      <formula1>Menu!$N$2:$N$3</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B17:B18">
-      <formula1>Menu!$H$2:$H$11</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B13:B13">
+      <formula1>Menu!$O$2:$O$20</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B19:B21">
-      <formula1>Menu!$I$2:$I$10</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B14:B14">
+      <formula1>Menu!$O$2:$O$20</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B15:B16">
+      <formula1>Menu!$E$2:$E$25</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B17:B19">
+      <formula1>Menu!$F$2:$F$13</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B20:B21">
+      <formula1>Menu!$G$2:$G$11</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B22:B24">
-      <formula1>Menu!$J$2:$J$34</formula1>
+      <formula1>Menu!$H$2:$H$10</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B30:B32">
-      <formula1>Menu!$K$2:$K$15</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B25:B27">
+      <formula1>Menu!$I$2:$I$34</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B33:B35">
+      <formula1>Menu!$J$2:$J$15</formula1>
     </dataValidation>
   </dataValidations>
 </worksheet>
@@ -3470,12 +3551,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K116"/>
+  <dimension ref="A1:R116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="60"/>
-    <col min="2" max="2" width="26"/>
-    <col min="4" max="11" width="34"/>
+    <col min="2" max="2" width="24"/>
+    <col min="4" max="10" width="30"/>
+    <col min="12" max="15" width="26"/>
+    <col min="17" max="18" width="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3491,42 +3574,67 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 - Base monitor</t>
+          <t xml:space="preserve">1 Base</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 - Sensors &amp; cartridges</t>
+          <t xml:space="preserve">3 EXO</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 - EXO modules &amp; accessories</t>
+          <t xml:space="preserve">4 Dock/G7</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 - Docking, charging &amp; G7 accessories</t>
+          <t xml:space="preserve">5 G6</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 - G6 accessories &amp; docks</t>
+          <t xml:space="preserve">6 Monitoring</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 - Monitoring &amp; data plans</t>
+          <t xml:space="preserve">7 Gas/consum</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">7 - Gas cylinders &amp; consumables</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8 - One-time services</t>
+          <t xml:space="preserve">8 One-time</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cartridge</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Combustible</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Oxygen</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Toxic sensors</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SensorMap name</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SensorMap SKU</t>
         </is>
       </c>
     </row>
@@ -3576,9 +3684,34 @@
           <t xml:space="preserve">- none -</t>
         </is>
       </c>
-      <c r="K2" s="8" t="inlineStr">
+      <c r="L2" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">- none -</t>
+        </is>
+      </c>
+      <c r="M2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- none -</t>
+        </is>
+      </c>
+      <c r="N2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- none -</t>
+        </is>
+      </c>
+      <c r="O2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- none -</t>
+        </is>
+      </c>
+      <c r="Q2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- none -</t>
+        </is>
+      </c>
+      <c r="R2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -3600,37 +3733,62 @@
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">NH3, high range NH3, NO2, O3, high range H2S or CO, COSH, Cl2, ClO2, C</t>
+          <t xml:space="preserve">Gas Expansion Module SO2, PID (SVXX)</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas Expansion Module SO2, PID (SVXX)</t>
+          <t xml:space="preserve">Rental service, beacon, daily rate</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental service, beacon, daily rate</t>
+          <t xml:space="preserve">Rental service, G6, H2S</t>
         </is>
       </c>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental service, G6, H2S</t>
+          <t xml:space="preserve">Custom update schedule, 5 minute frequency, daily rate</t>
         </is>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom update schedule, 5 minute frequency, daily rate</t>
+          <t xml:space="preserve">PTFE inlet filter</t>
         </is>
       </c>
       <c r="J3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">PTFE inlet filter</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="inlineStr">
-        <is>
           <t xml:space="preserve">Emergency order surcharge - call-out between 10 PM and 6 AM</t>
+        </is>
+      </c>
+      <c r="L3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diffusion cartridge (std sensors)</t>
+        </is>
+      </c>
+      <c r="M3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LEL-IR (infrared)</t>
+        </is>
+      </c>
+      <c r="N3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O2</t>
+        </is>
+      </c>
+      <c r="O3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H2S</t>
+        </is>
+      </c>
+      <c r="Q3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diffusion cartridge (std sensors)</t>
+        </is>
+      </c>
+      <c r="R3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RENT-CART-Q-XXXX</t>
         </is>
       </c>
     </row>
@@ -3652,37 +3810,57 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">CO2</t>
+          <t xml:space="preserve">Gas Expansion Module HF,NH3,SO2,PID (2ASV)</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas Expansion Module HF,NH3,SO2,PID (2ASV)</t>
+          <t xml:space="preserve">Rental service, G7 powerpack, daily rate</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental service, G7 powerpack, daily rate</t>
+          <t xml:space="preserve">Rental service, G6, CO</t>
         </is>
       </c>
       <c r="H4" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental service, G6, CO</t>
+          <t xml:space="preserve">Custom update schedule, 1 minute frequency, daily rate</t>
         </is>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom update schedule, 1 minute frequency, daily rate</t>
+          <t xml:space="preserve">Sintered metal pump stone, bag of 5</t>
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sintered metal pump stone, bag of 5</t>
-        </is>
-      </c>
-      <c r="K4" s="8" t="inlineStr">
-        <is>
           <t xml:space="preserve">Technician time, hourly, (cancellation, excess cleaning, etc.)</t>
+        </is>
+      </c>
+      <c r="L4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pumped cartridge (std sensors)</t>
+        </is>
+      </c>
+      <c r="M4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LEL-MPS (molecular property)</t>
+        </is>
+      </c>
+      <c r="O4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO</t>
+        </is>
+      </c>
+      <c r="Q4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pumped cartridge (std sensors)</t>
+        </is>
+      </c>
+      <c r="R4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RENT-CART-P-XXXX</t>
         </is>
       </c>
     </row>
@@ -3704,37 +3882,47 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">PID, HF</t>
+          <t xml:space="preserve">Gas Expansion Module H2,NH3,SO2,PID (6ASV)</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas Expansion Module H2,NH3,SO2,PID (6ASV)</t>
+          <t xml:space="preserve">Rental service, 5-bay charger, daily rate</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental service, 5-bay charger, daily rate</t>
+          <t xml:space="preserve">Rental service, G6, O2</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental service, G6, O2</t>
+          <t xml:space="preserve">Custom update schedule, 30 second frequency, daily rate</t>
         </is>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom update schedule, 30 second frequency, daily rate</t>
+          <t xml:space="preserve">Sintered metal pump stone</t>
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sintered metal pump stone</t>
-        </is>
-      </c>
-      <c r="K5" s="8" t="inlineStr">
-        <is>
           <t xml:space="preserve">Technician time, hourly, OT (callout)</t>
+        </is>
+      </c>
+      <c r="O5" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SO2</t>
+        </is>
+      </c>
+      <c r="Q5" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LEL-IR (infrared)</t>
+        </is>
+      </c>
+      <c r="R5" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -3756,37 +3944,47 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental service, diffusion cartridge, std. sensors, daily rate</t>
+          <t xml:space="preserve">Gas Expansion Module NH3,H2S,SO2 (AHSX)</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas Expansion Module NH3,H2S,SO2 (AHSX)</t>
+          <t xml:space="preserve">Rental service, 20-bay charger, daily rate</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental service, 20-bay charger, daily rate</t>
+          <t xml:space="preserve">Rental service, G6, SO2</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental service, G6, SO2</t>
+          <t xml:space="preserve">Custom update schedule, 10 second frequency, daily rate</t>
         </is>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom update schedule, 10 second frequency, daily rate</t>
+          <t xml:space="preserve">Whatman PTFE hydrophobic filter for 12" sample wand</t>
         </is>
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Whatman PTFE hydrophobic filter for 12" sample wand</t>
-        </is>
-      </c>
-      <c r="K6" s="8" t="inlineStr">
-        <is>
           <t xml:space="preserve">One time charge - as needed</t>
+        </is>
+      </c>
+      <c r="O6" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO-H</t>
+        </is>
+      </c>
+      <c r="Q6" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LEL-MPS (molecular property)</t>
+        </is>
+      </c>
+      <c r="R6" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -3808,37 +4006,47 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental service, pumped cartridge, std. sensors, daily rate</t>
+          <t xml:space="preserve">Gas Expansion Module H2,NH3,Cl2,PID (6ALV)</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas Expansion Module H2,NH3,Cl2,PID (6ALV)</t>
+          <t xml:space="preserve">Rental service, wall mount, 5-bay dock, loaded</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental service, wall mount, 5-bay dock, loaded</t>
+          <t xml:space="preserve">Rental service, G6 dock, daily rate</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental service, G6 dock, daily rate</t>
+          <t xml:space="preserve">Custom update schedule, 5 second frequency, daily rate</t>
         </is>
       </c>
       <c r="I7" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom update schedule, 5 second frequency, daily rate</t>
+          <t xml:space="preserve">Porex particulate filter for 12" sample wand</t>
         </is>
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Porex particulate filter for 12" sample wand</t>
-        </is>
-      </c>
-      <c r="K7" s="8" t="inlineStr">
-        <is>
           <t xml:space="preserve">Distributor owned device move fee - up to 50 units</t>
+        </is>
+      </c>
+      <c r="O7" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NH3</t>
+        </is>
+      </c>
+      <c r="Q7" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O2</t>
+        </is>
+      </c>
+      <c r="R7" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -3858,34 +4066,49 @@
           <t xml:space="preserve">Rental service, G7X, pump, daily rate</t>
         </is>
       </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gas Expansion Module H2,Cl2,HCN,PID (6LNV)</t>
+        </is>
+      </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas Expansion Module H2,Cl2,HCN,PID (6LNV)</t>
+          <t xml:space="preserve">Rental service, G7 dock, daily rate</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental service, G7 dock, daily rate</t>
+          <t xml:space="preserve">Rental Service, G6 Multi-Unit Charger, 5 Slots</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental Service, G6 Multi-Unit Charger, 5 Slots</t>
+          <t xml:space="preserve">Rental Service, Auto bump &amp; calibration, daily rate</t>
         </is>
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental Service, Auto bump &amp; calibration, daily rate</t>
+          <t xml:space="preserve">Lexan tube for 12" sample wand</t>
         </is>
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lexan tube for 12" sample wand</t>
-        </is>
-      </c>
-      <c r="K8" s="8" t="inlineStr">
-        <is>
           <t xml:space="preserve">Distributor owned device move fee - surcharge for units over 50</t>
+        </is>
+      </c>
+      <c r="O8" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High-range NH3</t>
+        </is>
+      </c>
+      <c r="Q8" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H2S</t>
+        </is>
+      </c>
+      <c r="R8" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -3905,34 +4128,49 @@
           <t xml:space="preserve">Rental service, G7X, standard Z cart, daily rate</t>
         </is>
       </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gas Expansion Module NH3,Cl2,HCN,PID (ALNV)</t>
+        </is>
+      </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas Expansion Module NH3,Cl2,HCN,PID (ALNV)</t>
+          <t xml:space="preserve">Rental service, G7 dock and regulator, daily rate</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental service, G7 dock and regulator, daily rate</t>
+          <t xml:space="preserve">Rental Service, G6 Multi-Unit Charger, 25 Slots</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental Service, G6 Multi-Unit Charger, 25 Slots</t>
+          <t xml:space="preserve">Rental Service, AlertLink, daily rate</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental Service, AlertLink, daily rate</t>
+          <t xml:space="preserve">Replacement o-ring for 12" sample wand</t>
         </is>
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Replacement o-ring for 12" sample wand</t>
-        </is>
-      </c>
-      <c r="K9" s="8" t="inlineStr">
-        <is>
           <t xml:space="preserve">Distributor owned device move fee - per-unit charge over 51</t>
+        </is>
+      </c>
+      <c r="O9" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO2</t>
+        </is>
+      </c>
+      <c r="Q9" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO</t>
+        </is>
+      </c>
+      <c r="R9" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -3952,34 +4190,49 @@
           <t xml:space="preserve">Rental service, G7X, single-gas, daily rate</t>
         </is>
       </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gas Expansion Module HF, H2, HCN (26NX)</t>
+        </is>
+      </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas Expansion Module HF, H2, HCN (26NX)</t>
+          <t xml:space="preserve">Rental service, demand flow regulator also suitable for sticky gases</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental service, demand flow regulator also suitable for sticky gases</t>
+          <t xml:space="preserve">Rental service, G6 calibration kit - tubing, cal cap</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental service, G6 calibration kit - tubing, cal cap</t>
+          <t xml:space="preserve">Rental Service, Blackline 24/7 live monitoring, daily rate</t>
         </is>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental Service, Blackline 24/7 live monitoring, daily rate</t>
+          <t xml:space="preserve">Replacement gasket for 12" sample wand</t>
         </is>
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Replacement gasket for 12" sample wand</t>
-        </is>
-      </c>
-      <c r="K10" s="8" t="inlineStr">
-        <is>
           <t xml:space="preserve">Training, Daily, at Blackline Facility</t>
+        </is>
+      </c>
+      <c r="O10" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O3</t>
+        </is>
+      </c>
+      <c r="Q10" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SO2</t>
+        </is>
+      </c>
+      <c r="R10" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -3999,29 +4252,44 @@
           <t xml:space="preserve">Rental service, G7 bridge, daily rate</t>
         </is>
       </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gas Expansion Module HF,NH3,Cl2,PID (2ALV)</t>
+        </is>
+      </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas Expansion Module HF,NH3,Cl2,PID (2ALV)</t>
+          <t xml:space="preserve">Rental service, fixed flow regulator</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rental service, fixed flow regulator</t>
-        </is>
-      </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
           <t xml:space="preserve">Rental service, G6 charge clip, block, and cable</t>
         </is>
       </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tubing 2' tygon</t>
+        </is>
+      </c>
       <c r="J11" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tubing 2' tygon</t>
-        </is>
-      </c>
-      <c r="K11" s="8" t="inlineStr">
-        <is>
           <t xml:space="preserve">Training, 1 day, at customer facility</t>
+        </is>
+      </c>
+      <c r="O11" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High-range H2S</t>
+        </is>
+      </c>
+      <c r="Q11" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO-H</t>
+        </is>
+      </c>
+      <c r="R11" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Premium Sensors - Daily</t>
         </is>
       </c>
     </row>
@@ -4041,24 +4309,39 @@
           <t xml:space="preserve">Rental service, EXO, daily rate</t>
         </is>
       </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gas Expansion Module NH3,H2S,Cl2,PID (AHLV)</t>
+        </is>
+      </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas Expansion Module NH3,H2S,Cl2,PID (AHLV)</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
           <t xml:space="preserve">Rental service, fixed flow regulator for sticky gases</t>
         </is>
       </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tubing 2' teflon</t>
+        </is>
+      </c>
       <c r="J12" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tubing 2' teflon</t>
-        </is>
-      </c>
-      <c r="K12" s="8" t="inlineStr">
-        <is>
           <t xml:space="preserve">Training, 2 days, at customer facility</t>
+        </is>
+      </c>
+      <c r="O12" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High-range CO</t>
+        </is>
+      </c>
+      <c r="Q12" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NH3</t>
+        </is>
+      </c>
+      <c r="R12" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Premium Sensors - Daily</t>
         </is>
       </c>
     </row>
@@ -4078,24 +4361,39 @@
           <t xml:space="preserve">Rental service, EXO, pump module, daily rate</t>
         </is>
       </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gas Expansion Module O3,H2,Cl2,SO2 (EHLS)</t>
+        </is>
+      </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas Expansion Module O3,H2,Cl2,SO2 (EHLS)</t>
-        </is>
-      </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
           <t xml:space="preserve">Rental service, handheld sample wand, 12", with filters</t>
         </is>
       </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tubing 10' tygon</t>
+        </is>
+      </c>
       <c r="J13" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tubing 10' tygon</t>
-        </is>
-      </c>
-      <c r="K13" s="8" t="inlineStr">
-        <is>
           <t xml:space="preserve">Training, 3 days, at customer facility</t>
+        </is>
+      </c>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">COSH</t>
+        </is>
+      </c>
+      <c r="Q13" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High-range NH3</t>
+        </is>
+      </c>
+      <c r="R13" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Premium Sensors - Daily</t>
         </is>
       </c>
     </row>
@@ -4115,19 +4413,34 @@
           <t xml:space="preserve">Rental service, EXO, satellite module, daily rate</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Rental service, EXO, universal mount, daily rate</t>
         </is>
       </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tubing 10' teflon</t>
+        </is>
+      </c>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tubing 10' teflon</t>
-        </is>
-      </c>
-      <c r="K14" s="8" t="inlineStr">
-        <is>
           <t xml:space="preserve">Training, 4 days, at customer facility</t>
+        </is>
+      </c>
+      <c r="O14" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cl2</t>
+        </is>
+      </c>
+      <c r="Q14" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO2</t>
+        </is>
+      </c>
+      <c r="R14" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Premium Sensors - Daily</t>
         </is>
       </c>
     </row>
@@ -4147,19 +4460,34 @@
           <t xml:space="preserve">Rental service, EXO, translator, daily</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Rental service, UMK gas cylinder bracket</t>
         </is>
       </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tubing 50' tygon</t>
+        </is>
+      </c>
       <c r="J15" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tubing 50' tygon</t>
-        </is>
-      </c>
-      <c r="K15" s="8" t="inlineStr">
-        <is>
           <t xml:space="preserve">Training, 5 days, at customer facility</t>
+        </is>
+      </c>
+      <c r="O15" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ClO2</t>
+        </is>
+      </c>
+      <c r="Q15" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O3</t>
+        </is>
+      </c>
+      <c r="R15" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Premium Sensors - Daily</t>
         </is>
       </c>
     </row>
@@ -4174,14 +4502,29 @@
           <t xml:space="preserve">RENT-EX8-GEM-01</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Rental service, auto bump and calibration kit (complete bundle)</t>
         </is>
       </c>
-      <c r="J16" s="8" t="inlineStr">
+      <c r="I16" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Tubing 50' teflon</t>
+        </is>
+      </c>
+      <c r="O16" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HCN</t>
+        </is>
+      </c>
+      <c r="Q16" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High-range H2S</t>
+        </is>
+      </c>
+      <c r="R16" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Premium Sensors - Daily</t>
         </is>
       </c>
     </row>
@@ -4196,14 +4539,29 @@
           <t xml:space="preserve">RENT-EX8-GEM-02</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Rental service, EXO, hanging mount, daily rate</t>
         </is>
       </c>
-      <c r="J17" s="8" t="inlineStr">
+      <c r="I17" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Tubing 100' tygon, large diameter</t>
+        </is>
+      </c>
+      <c r="O17" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H2</t>
+        </is>
+      </c>
+      <c r="Q17" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High-range CO</t>
+        </is>
+      </c>
+      <c r="R17" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Premium Sensors - Daily</t>
         </is>
       </c>
     </row>
@@ -4218,14 +4576,29 @@
           <t xml:space="preserve">RENT-EX8-GEM-03</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Rental service, EXO, solar panel kit, daily rate</t>
         </is>
       </c>
-      <c r="J18" s="8" t="inlineStr">
+      <c r="I18" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">G7 pump particulate filters, 10</t>
+        </is>
+      </c>
+      <c r="O18" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO2</t>
+        </is>
+      </c>
+      <c r="Q18" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">COSH</t>
+        </is>
+      </c>
+      <c r="R18" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Premium Sensors - Daily</t>
         </is>
       </c>
     </row>
@@ -4240,14 +4613,29 @@
           <t xml:space="preserve">RENT-EX8-GEM-04</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Rental service, G7 EXO, siren kit, daily rate</t>
         </is>
       </c>
-      <c r="J19" s="8" t="inlineStr">
+      <c r="I19" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">G7 single-gas calibration cap</t>
+        </is>
+      </c>
+      <c r="O19" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PID</t>
+        </is>
+      </c>
+      <c r="Q19" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cl2</t>
+        </is>
+      </c>
+      <c r="R19" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Premium Sensors - Daily</t>
         </is>
       </c>
     </row>
@@ -4262,14 +4650,29 @@
           <t xml:space="preserve">RENT-EX8-GEM-11</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Rental service, EXO, replacement battery, daily rate</t>
         </is>
       </c>
-      <c r="J20" s="8" t="inlineStr">
+      <c r="I20" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">G7 multi-gas calibration cap</t>
+        </is>
+      </c>
+      <c r="O20" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HF</t>
+        </is>
+      </c>
+      <c r="Q20" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ClO2</t>
+        </is>
+      </c>
+      <c r="R20" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Premium Sensors - Daily</t>
         </is>
       </c>
     </row>
@@ -4284,14 +4687,24 @@
           <t xml:space="preserve">RENT-EX8-GEM-05</t>
         </is>
       </c>
-      <c r="F21" s="8" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Rental service, EXO, survey tripod, daily rate</t>
         </is>
       </c>
-      <c r="J21" s="8" t="inlineStr">
+      <c r="I21" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">G6 replacement sensor cap</t>
+        </is>
+      </c>
+      <c r="Q21" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HCN</t>
+        </is>
+      </c>
+      <c r="R21" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Premium Sensors - Daily</t>
         </is>
       </c>
     </row>
@@ -4306,14 +4719,24 @@
           <t xml:space="preserve">RENT-EX8-GEM-06</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Rental service, EXO, standoff (low tripod), daily rate</t>
         </is>
       </c>
-      <c r="J22" s="8" t="inlineStr">
+      <c r="I22" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">34L Gas Cylinder, H2S 25ppm/CO 100ppm/CH4 50%LEL/O2 18%</t>
+        </is>
+      </c>
+      <c r="Q22" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H2</t>
+        </is>
+      </c>
+      <c r="R22" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Premium Sensors - Daily</t>
         </is>
       </c>
     </row>
@@ -4328,14 +4751,24 @@
           <t xml:space="preserve">RENT-EX8-GEM-07</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Rental service, EXO, safety tether, daily rate</t>
         </is>
       </c>
-      <c r="J23" s="8" t="inlineStr">
+      <c r="I23" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">116L Gas Cylinder, H2S 25ppm/CO 100ppm/CH4 50%LEL/O2 18%</t>
+        </is>
+      </c>
+      <c r="Q23" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO2</t>
+        </is>
+      </c>
+      <c r="R23" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Advanced Sensor - Daily</t>
         </is>
       </c>
     </row>
@@ -4350,14 +4783,24 @@
           <t xml:space="preserve">RENT-EX8-GEM-12</t>
         </is>
       </c>
-      <c r="F24" s="8" t="inlineStr">
+      <c r="E24" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Rental service, EXO, carrying case, daily rate</t>
         </is>
       </c>
-      <c r="J24" s="8" t="inlineStr">
+      <c r="I24" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">116L Gas Cylinder, SO2 10ppm, Balance air</t>
+        </is>
+      </c>
+      <c r="Q24" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PID</t>
+        </is>
+      </c>
+      <c r="R24" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VOC/HF Sensor - Daily</t>
         </is>
       </c>
     </row>
@@ -4372,14 +4815,24 @@
           <t xml:space="preserve">RENT-EX8-GEM-09</t>
         </is>
       </c>
-      <c r="F25" s="8" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Rental service, EXO, fast charger</t>
         </is>
       </c>
-      <c r="J25" s="8" t="inlineStr">
+      <c r="I25" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">58L Gas Cylinder, NH3 50ppm, Balance air</t>
+        </is>
+      </c>
+      <c r="Q25" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HF</t>
+        </is>
+      </c>
+      <c r="R25" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VOC/HF Sensor - Daily</t>
         </is>
       </c>
     </row>
@@ -4394,7 +4847,7 @@
           <t xml:space="preserve">RENT-EX8-GEM-08</t>
         </is>
       </c>
-      <c r="J26" s="8" t="inlineStr">
+      <c r="I26" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">116L Gas Cylinder, NH3 50ppm, Balance air</t>
         </is>
@@ -4411,7 +4864,7 @@
           <t xml:space="preserve">Premium Sensors - Daily</t>
         </is>
       </c>
-      <c r="J27" s="8" t="inlineStr">
+      <c r="I27" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">58L Gas Cylinder, Cl2 5ppm, Balance air</t>
         </is>
@@ -4428,7 +4881,7 @@
           <t xml:space="preserve">Advanced Sensor - Daily</t>
         </is>
       </c>
-      <c r="J28" s="8" t="inlineStr">
+      <c r="I28" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">58L Gas Cylinder, NO2, 10 ppm, Balance air</t>
         </is>
@@ -4445,7 +4898,7 @@
           <t xml:space="preserve">VOC/HF Sensor - Daily</t>
         </is>
       </c>
-      <c r="J29" s="8" t="inlineStr">
+      <c r="I29" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">116L Gas Cylinder, NO2, 10 ppm, Balance air</t>
         </is>
@@ -4462,7 +4915,7 @@
           <t xml:space="preserve">RENT-CART-Q-XXXX</t>
         </is>
       </c>
-      <c r="J30" s="8" t="inlineStr">
+      <c r="I30" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">116L Gas Cylinder, HCN 10 ppm, Balance air</t>
         </is>
@@ -4479,7 +4932,7 @@
           <t xml:space="preserve">RENT-CART-P-XXXX</t>
         </is>
       </c>
-      <c r="J31" s="8" t="inlineStr">
+      <c r="I31" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">58L Gas Cylinder, CO2 5000 ppm, Balance air</t>
         </is>
@@ -4496,7 +4949,7 @@
           <t xml:space="preserve">RENT-BEACON</t>
         </is>
       </c>
-      <c r="J32" s="8" t="inlineStr">
+      <c r="I32" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">58L Gas Cylinder, Isobutylene 100ppm, Balance air</t>
         </is>
@@ -4513,7 +4966,7 @@
           <t xml:space="preserve">RENT-ACC-G7-PWRPAC-NA</t>
         </is>
       </c>
-      <c r="J33" s="8" t="inlineStr">
+      <c r="I33" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">116L Gas Cylinder, Isobutylene 100ppm, Balance air</t>
         </is>
@@ -4530,7 +4983,7 @@
           <t xml:space="preserve">RENT-ACC-CHG-PNL-5-NA</t>
         </is>
       </c>
-      <c r="J34" s="8" t="inlineStr">
+      <c r="I34" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Gas, 10AL Gas Cylinder, UN1002 Air, 103L</t>
         </is>

</xml_diff>